<commit_message>
Add measurement report workbook analysis
</commit_message>
<xml_diff>
--- a/measurements/24/Filled_2D_sections/coronal/week24_coronal_Batch_Allmarks.xlsx
+++ b/measurements/24/Filled_2D_sections/coronal/week24_coronal_Batch_Allmarks.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Analysis" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -137,6 +138,211 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>15</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>15</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>15</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>15</col>
+      <colOff>0</colOff>
+      <row>67</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4953000" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>35</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5905500" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2055,4 +2261,1277 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Workbook Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Workbook</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>week24_coronal_Batch_Allmarks.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Axis</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>coronal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Slice rows analyzed</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>When a sulcus class count exceeds 3, approximate raw sulcus values are reconstructed from count + min/max/mean for summary stats and boxplots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Core Metric Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1597.862811791383</v>
+      </c>
+      <c r="D10" t="n">
+        <v>36.15720694602083</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1499.886621315193</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1626.303854875283</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>perimeter</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" t="n">
+        <v>211.2218989218984</v>
+      </c>
+      <c r="D11" t="n">
+        <v>6.955162045739264</v>
+      </c>
+      <c r="E11" t="n">
+        <v>198.369372118087</v>
+      </c>
+      <c r="F11" t="n">
+        <v>219.3894365287962</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LGI</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.148838685444346</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.01845798466230702</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.118375509112735</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.173701531027829</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Compactness</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4508924683129573</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.02133143268059214</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.4226168541957873</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.4874906462988245</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rounded Sulcus Counts Per Slice</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sulci_count</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Primary_count</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Secondary_count</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Tertiary_count</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Unclassified_count</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Sulci_count_rounded</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Primary_count_rounded</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Secondary_count_rounded</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Tertiary_count_rounded</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Unclassified_count_rounded</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>band_axis1_s00_idx0089.png</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>band_axis1_s01_idx0091.png</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>band_axis1_s02_idx0092.png</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>band_axis1_s03_idx0093.png</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>band_axis1_s04_idx0095.png</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>band_axis1_s05_idx0096.png</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>band_axis1_s06_idx0097.png</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>band_axis1_s07_idx0099.png</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>band_axis1_s08_idx0100.png</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>band_axis1_s09_idx0101.png</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>band_axis1_s10_idx0103.png</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>band_axis1_s11_idx0104.png</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>band_axis1_s12_idx0105.png</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>band_axis1_s13_idx0107.png</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>4</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>band_axis1_s14_idx0108.png</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>4</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>band_axis1_s15_idx0109.png</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>band_axis1_s16_idx0111.png</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>4</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>band_axis1_s17_idx0112.png</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>4</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>band_axis1_s18_idx0113.png</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>band_axis1_s19_idx0114.png</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Rounded Sulcus Count Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sulci_count_rounded</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>20</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.4442616583193193</v>
+      </c>
+      <c r="E40" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Primary_count_rounded</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>20</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.3663475485325233</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Secondary_count_rounded</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>20</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.6386663736585051</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Tertiary_count_rounded</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>20</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.6708203932499369</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Unclassified_count_rounded</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>20</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sulcus Value Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>primary_sulcus_values</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>23</v>
+      </c>
+      <c r="C48" t="n">
+        <v>10.52431094720497</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.6253671107732552</v>
+      </c>
+      <c r="E48" t="n">
+        <v>8.844866071428571</v>
+      </c>
+      <c r="F48" t="n">
+        <v>11.25</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>secondary_sulcus_values</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>55</v>
+      </c>
+      <c r="C49" t="n">
+        <v>6.151041666666665</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.059151403376981</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3.078497023809524</v>
+      </c>
+      <c r="F49" t="n">
+        <v>7.756696428571428</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>tertiary_sulcus_values</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>7</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1.193930697278911</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.6536833703925623</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.8147321428571428</v>
+      </c>
+      <c r="F50" t="n">
+        <v>2.514880952380952</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>unclassified_sulcus_values</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>